<commit_message>
Voeg beantwoording en tussenbericht kolommen toe aan schriftelijke vragen
Parse de 'Relatie met' sectie op de detailpagina om gerelateerde
Brieven B&W documenten te vinden. Volgt elk gerelateerd item om de
PDF-URL op te halen. Onderscheidt tussenberichten (titel start met
'Tussenbericht') van definitieve beantwoording.

Fix: html.unescape() voor 'Brieven B&W' entiteit matching.
Test: 100 records → 35 beantwoordingen, 16 tussenberichten gevonden.

https://claude.ai/code/session_01Pt5DG8UgHAMFs55hwQTGmN
</commit_message>
<xml_diff>
--- a/schriftelijke_vragen.xlsx
+++ b/schriftelijke_vragen.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Schriftelijke vragen" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schriftelijke vragen'!$A$1:$L$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schriftelijke vragen'!$A$1:$P$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:P101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -468,9 +468,13 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="80" customWidth="1" min="8" max="8"/>
     <col width="50" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="100" customWidth="1" min="11" max="11"/>
-    <col width="100" customWidth="1" min="12" max="12"/>
+    <col width="80" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="80" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="100" customWidth="1" min="15" max="15"/>
+    <col width="100" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -521,15 +525,35 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Tussenbericht(en)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Tussenbericht URL(s)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Beantwoording</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Beantwoording URL</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Aantal bijlagen</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Bijlagen</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Bijlage URLs</t>
         </is>
@@ -577,11 +601,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/67ba1357-cfce-4d5c-898c-466fd5cbd1f9?documentId=556220e0-8125-42a3-b1e3-447abc9edca9</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -625,11 +653,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/47e6de16-04a4-41e1-bae1-30ee3f99e729?documentId=25757aed-f8b4-4693-b682-fc10a4844918</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -673,11 +705,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/b01e1c3d-a774-4f86-bb37-808d27fb7c2a?documentId=870c26fa-46c7-4a59-bea0-de14e52bff32</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -721,11 +757,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/b8e87a29-155d-4c13-8227-d2df93caac47?documentId=520492bd-cd39-4f88-b94f-cf516936b16c</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -769,11 +809,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/51db4d44-8fb4-47b2-b4f3-441e5a92c88c?documentId=4f5a59cf-c3a2-4380-99ac-c768121f8c78</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -817,11 +861,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/4e8669d0-15e3-41d2-9422-d529a54c0edb?documentId=16845c71-b626-42c1-9dbb-5e445ee2403f</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -865,11 +913,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/a75f31aa-72f4-409e-a5ce-9e9e1fae8c40?documentId=c8e06df3-022b-45b1-b9ab-3602d403d051</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -913,11 +965,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/2ff66b65-75cf-45be-b2de-0da35f283094?documentId=692186a0-b83f-41a7-a43e-013a6f8b436d</t>
         </is>
       </c>
-      <c r="J9" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="2" t="inlineStr"/>
+      <c r="P9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -961,11 +1017,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/adcf8dd8-e2cb-4f40-884e-472116779bab?documentId=dbb442d3-ce24-4cbb-a835-dec5c51706a5</t>
         </is>
       </c>
-      <c r="J10" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1009,11 +1069,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/ceb344ad-8d62-4d36-ac58-a37988f00d32?documentId=6af28b72-d896-43fb-b8f4-0a370a5c8bf6</t>
         </is>
       </c>
-      <c r="J11" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1057,11 +1121,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/8a0156a8-a201-45b4-b404-e6dfe3ba6a2b?documentId=de84eba0-5a6f-437c-9e71-62bc6774e78e</t>
         </is>
       </c>
-      <c r="J12" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1105,11 +1173,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/51752b56-2cf1-4237-9193-f306dee3d7de?documentId=d33bc961-ba0f-40d6-aa54-b0d2953ebe88</t>
         </is>
       </c>
-      <c r="J13" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="2" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1153,11 +1225,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/93bb4784-45a9-407d-a7ce-00797d6f2dea?documentId=dbc7b334-4bfa-4134-89a2-fb59f832d816</t>
         </is>
       </c>
-      <c r="J14" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1201,11 +1277,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/ef49609f-e7da-4923-9845-d2e3a6a90ce8?documentId=2781d40b-6d4b-42a1-a71e-d21814619780</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1249,11 +1329,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/12f7fd05-4085-4369-b06e-7499f819bdfc?documentId=f74cf7e8-9087-480b-b133-54a134038b14</t>
         </is>
       </c>
-      <c r="J16" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1297,11 +1381,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/00376bd0-65d9-4679-9dd3-b8ec316f5eb1?documentId=430cb7e4-df38-41a9-99c8-94a604d2075b</t>
         </is>
       </c>
-      <c r="J17" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1345,11 +1433,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/19c2cad2-da45-4393-a57e-bde5a52025a8?documentId=260884fe-532f-4ba9-b26b-338d13fdb490</t>
         </is>
       </c>
-      <c r="J18" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="2" t="inlineStr"/>
+      <c r="P18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1397,11 +1489,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/2ae24ea3-e738-443c-8c25-ba64276daaf4?documentId=96743168-d4be-4417-9c6f-a02050512e28</t>
         </is>
       </c>
-      <c r="J19" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001592] Beantwoording vragen Coskun over Deel concept vervoersplan 2027 voor de verkiezingen</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/c523cec4-6c8b-4433-8d67-51c5dd932fb0?documentId=42d17a26-9d7c-403b-bd5d-89a63aa6f585</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="2" t="inlineStr"/>
+      <c r="P19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1445,11 +1549,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/5d769eb4-b0b0-4cca-85b8-c3e41ddccd80?documentId=a90fe25c-5187-4c1f-ac2a-0b706287f89f</t>
         </is>
       </c>
-      <c r="J20" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="2" t="inlineStr"/>
+      <c r="P20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1493,11 +1601,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/cc8558c7-d8d9-445e-b84d-a0826b0d9199?documentId=d3e82d73-1899-43dc-a718-f327c62dbdad</t>
         </is>
       </c>
-      <c r="J21" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="2" t="inlineStr"/>
+      <c r="P21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1541,11 +1653,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/9d8a6dfc-cde7-40b9-8494-5017caa8c9df?documentId=a791148b-563a-4f02-9b3c-1f9ce06a79c3</t>
         </is>
       </c>
-      <c r="J22" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="2" t="inlineStr"/>
+      <c r="P22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1589,11 +1705,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/eabb5550-9a68-4428-a0dc-6ac385693cef?documentId=55168d5d-7ace-45a3-a325-c9e0f567abe6</t>
         </is>
       </c>
-      <c r="J23" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="2" t="inlineStr"/>
+      <c r="P23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1637,11 +1757,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/63b47650-0381-41e4-b5de-6273e6f7f309?documentId=26742bb1-8de1-41cb-84c8-a49dd04f6546</t>
         </is>
       </c>
-      <c r="J24" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="2" t="inlineStr"/>
+      <c r="P24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1685,11 +1809,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/e5dddbcd-eea2-4357-9c9b-cb10ef56a130?documentId=b3eea2f4-6953-428e-aaba-e66d57f0be59</t>
         </is>
       </c>
-      <c r="J25" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="2" t="inlineStr"/>
+      <c r="P25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1733,11 +1861,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/493a9f5c-c99e-47a3-b579-e78f83bd115d?documentId=52610e41-e64a-4573-aea5-f9ebaef3d418</t>
         </is>
       </c>
-      <c r="J26" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1781,11 +1913,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/07737743-a14e-4384-b0b2-13609210bc7d?documentId=2bed1d89-1917-4dc9-b505-68d787e6d55b</t>
         </is>
       </c>
-      <c r="J27" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1829,11 +1965,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/dd36a6aa-cfbb-4b5f-95eb-8dd022468e35?documentId=b200f66a-579e-4dad-b7cc-7a0c48759901</t>
         </is>
       </c>
-      <c r="J28" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1877,11 +2017,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/b99cb940-1487-4ee8-bb57-95e74c002c12?documentId=55702fc8-cabe-49b6-9315-84ce3dc3a7df</t>
         </is>
       </c>
-      <c r="J29" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J29" s="2" t="inlineStr"/>
       <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="2" t="inlineStr"/>
+      <c r="P29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1925,11 +2069,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/6afce375-f04b-4e2a-b62a-3d985ff7375b?documentId=c35f2a04-19d4-46b1-aa89-4f6c95548832</t>
         </is>
       </c>
-      <c r="J30" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="2" t="inlineStr"/>
+      <c r="P30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1973,11 +2121,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/efa02ab3-4d17-4397-a93e-dd2fed4bd9b5?documentId=c8bf522d-8345-43d1-b7cd-b07a4e525891</t>
         </is>
       </c>
-      <c r="J31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001665] Tussenbericht vragen Abrahamse over Windmolens Beneluxplein</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/6f78cd9b-cffa-4edc-a3a2-0f25f36c8526?documentId=82600b50-a0d9-4146-8117-1dc06a011fc9</t>
+        </is>
+      </c>
       <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr"/>
+      <c r="N31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="2" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2021,11 +2181,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/7b2c8eb7-fdd0-47e9-9ca0-bfe74d6ecb29?documentId=bae49be2-6764-4993-b9fd-719f2862ea8d</t>
         </is>
       </c>
-      <c r="J32" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J32" s="2" t="inlineStr"/>
       <c r="K32" s="2" t="inlineStr"/>
       <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="2" t="inlineStr"/>
+      <c r="P32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2073,11 +2237,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/68e9505e-be88-4d61-8672-1bc0db3ce5cc?documentId=fcf1ae07-d054-43b0-84de-8f4b959476fb</t>
         </is>
       </c>
-      <c r="J33" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J33" s="2" t="inlineStr"/>
       <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001601] Beantwoording vragen Becker en Rehim Zadeh over Aangekondigde taxistaking Taxibranche</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/483fe85d-56c8-4ff0-a03e-e16eb94edd62?documentId=38d41caf-8e52-4c28-8f17-37ac4246c3b8</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="2" t="inlineStr"/>
+      <c r="P33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2121,11 +2297,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/0276f430-9569-4c84-bfbe-02092a3d480d?documentId=67b70cd3-ae6d-4f8c-ab8c-ad0a38cea986</t>
         </is>
       </c>
-      <c r="J34" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr"/>
       <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="2" t="inlineStr"/>
+      <c r="P34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2169,11 +2349,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/ae993fc3-565c-47cd-b76c-e4b5d8c9848b?documentId=74258c11-d3ec-442e-810d-81b7d99e18f5</t>
         </is>
       </c>
-      <c r="J35" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J35" s="2" t="inlineStr"/>
       <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr"/>
+      <c r="N35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" s="2" t="inlineStr"/>
+      <c r="P35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2217,11 +2401,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/c8bf28aa-79ea-4eb0-8087-bd3528b49647?documentId=0f9694e5-d0c4-4284-bd5b-4339552fe471</t>
         </is>
       </c>
-      <c r="J36" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J36" s="2" t="inlineStr"/>
       <c r="K36" s="2" t="inlineStr"/>
       <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="2" t="inlineStr"/>
+      <c r="P36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2265,11 +2453,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/839df3d2-44f3-4659-8279-d4a1e9471b08?documentId=e3007173-5c08-46a9-b2fa-8d24b2999f9e</t>
         </is>
       </c>
-      <c r="J37" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J37" s="2" t="inlineStr"/>
       <c r="K37" s="2" t="inlineStr"/>
       <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr"/>
+      <c r="N37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="2" t="inlineStr"/>
+      <c r="P37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2313,11 +2505,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/b6b1b23d-168b-4567-9831-292297bbcbf0?documentId=284b248f-2d03-4c10-9ce8-072b077a0d1b</t>
         </is>
       </c>
-      <c r="J38" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="2" t="inlineStr"/>
+      <c r="P38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2361,11 +2557,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/8172f897-6b22-4dd6-a47d-858d8d40f9df?documentId=9ebfa68e-a087-4378-ae58-e819b9f86cfe</t>
         </is>
       </c>
-      <c r="J39" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J39" s="2" t="inlineStr"/>
       <c r="K39" s="2" t="inlineStr"/>
       <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr"/>
+      <c r="N39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="2" t="inlineStr"/>
+      <c r="P39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2409,11 +2609,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/7b36150b-5bb6-4e87-9045-f590ec4dc26c?documentId=55d73e9b-3d62-4843-8fa3-4efa2736d6f2</t>
         </is>
       </c>
-      <c r="J40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001254] Tussenbericht vragen Nunnely over Leven in het leegstaande Donner pand</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/38eda0f9-6fea-4950-b63b-795bbc193765?documentId=1d47eed6-3fea-47f6-b3c2-3727c9cc498d</t>
+        </is>
+      </c>
       <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="2" t="inlineStr"/>
+      <c r="P40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2457,11 +2669,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/03096c03-c818-472b-9c94-f9882c4c0bc9?documentId=7a4020b8-41b8-479e-ba0e-d23c2501291a</t>
         </is>
       </c>
-      <c r="J41" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J41" s="2" t="inlineStr"/>
       <c r="K41" s="2" t="inlineStr"/>
       <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr"/>
+      <c r="N41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="2" t="inlineStr"/>
+      <c r="P41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2509,11 +2725,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/17e718f6-3647-4839-bd86-81878ad9c1d0?documentId=c6cfd43b-093f-412c-9a1a-3c916f8f94bc</t>
         </is>
       </c>
-      <c r="J42" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr"/>
-      <c r="L42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001209] Beantwoording vragen Roskam over de Diversiteitskalender 2026</t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/f5471aff-ec53-4872-81e8-465dce85bcd1?documentId=ba36706a-6b27-4cf7-a010-965ea8499e00</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" s="2" t="inlineStr"/>
+      <c r="P42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2561,11 +2789,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/9a6988f8-9e5d-4ded-99df-b2336ec249f1?documentId=6fa85e83-c516-41cf-ae01-ebfd3c7fc57b</t>
         </is>
       </c>
-      <c r="J43" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J43" s="2" t="inlineStr"/>
       <c r="K43" s="2" t="inlineStr"/>
-      <c r="L43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000631] Beantwoording vragen Becker over het proces van mogelijke opvang in de voormalige Visus-kliniek</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/06bf5008-a15d-4a89-9e8f-3a85e8fd2f8d?documentId=ad8fb670-d838-48e0-b2b6-a97124ca5c36</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" s="2" t="inlineStr"/>
+      <c r="P43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2613,11 +2853,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/9407cbb6-b2fb-424b-aeb1-d91bd052ba01?documentId=7f0e5228-385a-4e69-8c96-680a9770609b</t>
         </is>
       </c>
-      <c r="J44" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J44" s="2" t="inlineStr"/>
       <c r="K44" s="2" t="inlineStr"/>
-      <c r="L44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001388] Beantwoording vragen Bruin over Een koopwoning &amp;#233;n ook sociale huur?</t>
+        </is>
+      </c>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/50844132-fce6-4823-b99d-563c6caff433?documentId=a18d25a1-61e4-4ce3-9642-74230d7a7a91</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" s="2" t="inlineStr"/>
+      <c r="P44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2665,11 +2917,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/d3d92033-88bf-4a9b-b2d5-701b212f7368?documentId=ab532e4f-095a-44a7-8e3e-df78fd1e45cb</t>
         </is>
       </c>
-      <c r="J45" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J45" s="2" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr"/>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001295] Beantwoording vragen Nunnely over meer ruimte voor MBO-studentenverenigingen</t>
+        </is>
+      </c>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/6b58d639-d3df-45f5-9b5b-1f7d737c2297?documentId=5b32e1f5-4056-484a-a989-a29296b91a17</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" s="2" t="inlineStr"/>
+      <c r="P45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2713,11 +2977,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/96dd6389-3cf6-4cbd-b25c-5bf327b85a1d?documentId=e8cb23a7-a827-487e-bed1-1ca0edbfde3e</t>
         </is>
       </c>
-      <c r="J46" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000325] Tussenbericht vragen Publieke kijklocaties tijdens het WK 2026 in Rotterdam</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/4b1a0a71-aa01-4df6-8ac8-212caf5b4593?documentId=cb9e3a8b-031d-4cbc-9df3-04619979d7b4</t>
+        </is>
+      </c>
       <c r="L46" s="2" t="inlineStr"/>
+      <c r="M46" s="2" t="inlineStr"/>
+      <c r="N46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" s="2" t="inlineStr"/>
+      <c r="P46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2761,11 +3037,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/78a31eb4-f0ee-4000-8af9-5f8cf75ebacd?documentId=bfa11ecc-952e-4234-a2fe-0f17183adeae</t>
         </is>
       </c>
-      <c r="J47" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J47" s="2" t="inlineStr"/>
       <c r="K47" s="2" t="inlineStr"/>
       <c r="L47" s="2" t="inlineStr"/>
+      <c r="M47" s="2" t="inlineStr"/>
+      <c r="N47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" s="2" t="inlineStr"/>
+      <c r="P47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2809,11 +3089,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/94f1dc48-75a9-4d5e-9822-8d5f962153b8?documentId=d719aa38-460c-46cd-b4e7-8a2d3bb865f0</t>
         </is>
       </c>
-      <c r="J48" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr"/>
+      <c r="M48" s="2" t="inlineStr"/>
+      <c r="N48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" s="2" t="inlineStr"/>
+      <c r="P48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2857,11 +3141,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/9d94c516-3f57-49d8-8a76-8214a36d9b98?documentId=d8b60ebe-a22e-4762-bf8b-6397c80e1392</t>
         </is>
       </c>
-      <c r="J49" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J49" s="2" t="inlineStr"/>
       <c r="K49" s="2" t="inlineStr"/>
       <c r="L49" s="2" t="inlineStr"/>
+      <c r="M49" s="2" t="inlineStr"/>
+      <c r="N49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O49" s="2" t="inlineStr"/>
+      <c r="P49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2905,11 +3193,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/2880be57-a3a5-4974-a03c-fb23da7d7899?documentId=98449f39-a1a2-4081-b81f-d1e305447fb6</t>
         </is>
       </c>
-      <c r="J50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001606] Tussenbericht vragen Bruin en Verhoef over onderverhuur sociale huur in Rotterdam: wat gebeurt er echt?</t>
+        </is>
+      </c>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/9c21d1ec-2273-40bc-8510-75d517d6b101?documentId=388ff657-7efa-4146-b554-7f29df1fa960</t>
+        </is>
+      </c>
       <c r="L50" s="2" t="inlineStr"/>
+      <c r="M50" s="2" t="inlineStr"/>
+      <c r="N50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" s="2" t="inlineStr"/>
+      <c r="P50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2953,11 +3253,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/548b9a21-52bc-424f-8fb7-a701104d8c9b?documentId=6d70567d-2646-4e7b-bd3b-6b5abeb8eadb</t>
         </is>
       </c>
-      <c r="J51" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J51" s="2" t="inlineStr"/>
       <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr"/>
+      <c r="M51" s="2" t="inlineStr"/>
+      <c r="N51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O51" s="2" t="inlineStr"/>
+      <c r="P51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3001,11 +3305,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/55e51a02-ade5-45f8-8d26-fd6758dd8a3d?documentId=6096d5ce-5cce-49bd-ab63-e1818eb3729f</t>
         </is>
       </c>
-      <c r="J52" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr"/>
       <c r="L52" s="2" t="inlineStr"/>
+      <c r="M52" s="2" t="inlineStr"/>
+      <c r="N52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O52" s="2" t="inlineStr"/>
+      <c r="P52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3053,11 +3361,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/55ded8a4-92a7-41a6-b074-c2e569b64c53?documentId=1bf7cd97-c3ab-41ac-99c0-55e8c4b6f93c</t>
         </is>
       </c>
-      <c r="J53" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J53" s="2" t="inlineStr"/>
       <c r="K53" s="2" t="inlineStr"/>
-      <c r="L53" s="2" t="inlineStr"/>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001167] Beantwoording vragen Abrahamse over Bewonersoverlast door verschuiving drijvend park Rijnhaven</t>
+        </is>
+      </c>
+      <c r="M53" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/fd2e3566-e96d-4ed7-9bfd-18cec9127bfa?documentId=dfacf35d-15a4-4b14-bfaf-b5d1172c5b55</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O53" s="2" t="inlineStr"/>
+      <c r="P53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3101,11 +3421,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/4f198de8-59db-4360-a165-5e4bc419055e?documentId=52cfb062-10c6-4b43-a699-a7a92fa62946</t>
         </is>
       </c>
-      <c r="J54" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr"/>
       <c r="L54" s="2" t="inlineStr"/>
+      <c r="M54" s="2" t="inlineStr"/>
+      <c r="N54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" s="2" t="inlineStr"/>
+      <c r="P54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3153,11 +3477,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/50a916f0-21b8-45e9-a09c-5a09cfa4d013?documentId=f209d155-2b2f-4bc4-abfd-335163bfea10</t>
         </is>
       </c>
-      <c r="J55" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J55" s="2" t="inlineStr"/>
       <c r="K55" s="2" t="inlineStr"/>
-      <c r="L55" s="2" t="inlineStr"/>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001750] Beantwoording vragen de Waard over Aan de buis genageld</t>
+        </is>
+      </c>
+      <c r="M55" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/27105e20-c966-486c-af9c-945f4daa4160?documentId=262b88a2-4655-4f80-ae2f-80a9a613f0f7</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" s="2" t="inlineStr"/>
+      <c r="P55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3205,11 +3541,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/a663b37d-5dcf-40c7-9f68-694080ac06f9?documentId=19510e01-d4b5-41ef-801d-26328886a7b5</t>
         </is>
       </c>
-      <c r="J56" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J56" s="2" t="inlineStr"/>
       <c r="K56" s="2" t="inlineStr"/>
-      <c r="L56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000774] Beantwoording vragen Nunnely ea over Problemen bij adoptie en naamswijziging</t>
+        </is>
+      </c>
+      <c r="M56" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/dfbad81c-7df9-4972-b3a3-341440b32a75?documentId=71e609c5-b3d2-4438-a6c3-1625ca87271c</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="2" t="inlineStr"/>
+      <c r="P56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3253,11 +3601,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/33730069-9df9-4d76-a17b-4db5d62b73f0?documentId=f9a3788a-8a79-4ac4-b1bd-95a38b80e8ac</t>
         </is>
       </c>
-      <c r="J57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000767] Tussenbericht vragen van Groningen over ondergronds bankieren in Prada-toko- hoe voorkomt Rotterdam dat jongeren worden meegesleurd</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/86a88f9d-9e7d-461d-ad66-0f1b6bac8436?documentId=3a16a2e8-8162-4c5c-8778-4797851a2735</t>
+        </is>
+      </c>
       <c r="L57" s="2" t="inlineStr"/>
+      <c r="M57" s="2" t="inlineStr"/>
+      <c r="N57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" s="2" t="inlineStr"/>
+      <c r="P57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3305,11 +3665,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/cc9dba41-4df1-4928-9f14-b8b73d664f66?documentId=47772239-9a22-4e08-b2f7-79c7c28c2ec6</t>
         </is>
       </c>
-      <c r="J58" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J58" s="2" t="inlineStr"/>
       <c r="K58" s="2" t="inlineStr"/>
-      <c r="L58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001163] Beantwoording vragen Coskun over Carnisse wordt onbetaalbaar gemaakt</t>
+        </is>
+      </c>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/6f55d6a7-37cd-4a58-8b74-56fba1c4fa9f?documentId=5706c4e6-b86e-47cc-8f5e-5c95046cc443</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" s="2" t="inlineStr"/>
+      <c r="P58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3353,11 +3725,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/fd301eef-d89d-4817-beb0-3915d1c6bee5?documentId=4eb8cda1-1519-4636-9144-30f23ee59d46</t>
         </is>
       </c>
-      <c r="J59" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J59" s="2" t="inlineStr"/>
       <c r="K59" s="2" t="inlineStr"/>
       <c r="L59" s="2" t="inlineStr"/>
+      <c r="M59" s="2" t="inlineStr"/>
+      <c r="N59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O59" s="2" t="inlineStr"/>
+      <c r="P59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3405,11 +3781,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/28482c96-a2a6-4063-b738-1088c928f042?documentId=0c713d18-4927-489e-aae9-85def2cfbfd2</t>
         </is>
       </c>
-      <c r="J60" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J60" s="2" t="inlineStr"/>
       <c r="K60" s="2" t="inlineStr"/>
-      <c r="L60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000629] Beantwoording vragen Crielaard over KNVB - campus niet naar Rotterdam</t>
+        </is>
+      </c>
+      <c r="M60" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/7f6770f4-cc2b-417e-b00b-08b8ad6aa267?documentId=fd6f9042-9612-43a0-a373-d3d1116d3a09</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O60" s="2" t="inlineStr"/>
+      <c r="P60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3453,11 +3841,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/3eb8b4af-72db-4aeb-93fa-fe482792375f?documentId=135032cc-9e54-4e13-8435-e17efffcd9a0</t>
         </is>
       </c>
-      <c r="J61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001145] Tussenbericht vragen Akhatab over Zwemmen voor iedere Rotterdammer toegankelijk houden</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/acaf1471-2fcb-4996-8e61-f3f53911133f?documentId=ffd198b7-1bee-4257-b6ca-77535889d0bf</t>
+        </is>
+      </c>
       <c r="L61" s="2" t="inlineStr"/>
+      <c r="M61" s="2" t="inlineStr"/>
+      <c r="N61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" s="2" t="inlineStr"/>
+      <c r="P61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3501,11 +3901,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/944a25a0-cb51-4da9-955a-c5f05b85b64b?documentId=18a874ed-84c2-4cee-a16a-14b91eec0121</t>
         </is>
       </c>
-      <c r="J62" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J62" s="2" t="inlineStr"/>
       <c r="K62" s="2" t="inlineStr"/>
       <c r="L62" s="2" t="inlineStr"/>
+      <c r="M62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O62" s="2" t="inlineStr"/>
+      <c r="P62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3553,11 +3957,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/aefae31b-3c4f-4040-ae41-0cfb66b712a7?documentId=899ff949-f5b9-4112-877f-11d82c3b5abc</t>
         </is>
       </c>
-      <c r="J63" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J63" s="2" t="inlineStr"/>
       <c r="K63" s="2" t="inlineStr"/>
-      <c r="L63" s="2" t="inlineStr"/>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000722] Beantwoording vragen Verhoef en Crielaard over Kwaaitaalvloeren in sportcomplexen</t>
+        </is>
+      </c>
+      <c r="M63" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/c8eb5f8f-8f03-4aa1-934d-9b047a90881e?documentId=eaf65cca-3e07-41c8-bf49-1d82be382c3d</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O63" s="2" t="inlineStr"/>
+      <c r="P63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3601,11 +4017,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/6cdb8e37-1df3-43cd-bdc2-8ca0a66224c8?documentId=80643572-9e9c-42bd-859f-23e2eecc6fd6</t>
         </is>
       </c>
-      <c r="J64" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000018] Tussenbericht vragen Dekkers ea over Short stay onder de loep</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/b396e5f0-770d-4dc0-90ae-45fd9408a169?documentId=339b4f38-f496-4f6d-a937-7d607d21b699</t>
+        </is>
+      </c>
       <c r="L64" s="2" t="inlineStr"/>
+      <c r="M64" s="2" t="inlineStr"/>
+      <c r="N64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O64" s="2" t="inlineStr"/>
+      <c r="P64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3649,11 +4077,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/d124b0b7-2238-4dc0-a6a1-5ac73be6dc96?documentId=ffe0f2c1-e912-4d21-a5e2-07433c0cd0f0</t>
         </is>
       </c>
-      <c r="J65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000083] Tussenbericht vragen Coskun ov er N+P van Heijplaat naar Rozenburg</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/9c1dddda-bbd0-4c3d-a2c1-652df1fd5cad?documentId=41d319b6-4127-46db-8c1c-50d647b04964</t>
+        </is>
+      </c>
       <c r="L65" s="2" t="inlineStr"/>
+      <c r="M65" s="2" t="inlineStr"/>
+      <c r="N65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O65" s="2" t="inlineStr"/>
+      <c r="P65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3697,11 +4137,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/f2f6048f-5b60-4e41-a20f-e0bc195286e9?documentId=8f0a8bfd-871c-4d83-bcd2-77b2d38c0dba</t>
         </is>
       </c>
-      <c r="J66" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J66" s="2" t="inlineStr"/>
       <c r="K66" s="2" t="inlineStr"/>
       <c r="L66" s="2" t="inlineStr"/>
+      <c r="M66" s="2" t="inlineStr"/>
+      <c r="N66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O66" s="2" t="inlineStr"/>
+      <c r="P66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3745,11 +4189,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/d79d2d95-c41d-4f35-a70f-3dd873a468b4?documentId=9f8c6008-614e-4412-94e7-cca81ef92ba9</t>
         </is>
       </c>
-      <c r="J67" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J67" s="2" t="inlineStr"/>
       <c r="K67" s="2" t="inlineStr"/>
       <c r="L67" s="2" t="inlineStr"/>
+      <c r="M67" s="2" t="inlineStr"/>
+      <c r="N67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O67" s="2" t="inlineStr"/>
+      <c r="P67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3797,11 +4245,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/22e81dd9-eeeb-4d2d-b46b-ec22e4e3d9b0?documentId=6e71c671-2e1d-4a3b-ab62-c1cc21c0e211</t>
         </is>
       </c>
-      <c r="J68" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J68" s="2" t="inlineStr"/>
       <c r="K68" s="2" t="inlineStr"/>
-      <c r="L68" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000421] Beantwoording vragen Verhoef en Bruin over Brandveiligheid bij hoogbouw</t>
+        </is>
+      </c>
+      <c r="M68" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/ae4a7388-ce55-470b-88d5-6250ea72a4c9?documentId=13ac84aa-4119-4cc0-bf06-853fcb5108cd</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O68" s="2" t="inlineStr"/>
+      <c r="P68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -3849,11 +4309,31 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/05eadbf2-be64-4f9f-878a-c39aa7ed1f14?documentId=b8db58a7-3887-472f-848d-988187206df4</t>
         </is>
       </c>
-      <c r="J69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K69" s="2" t="inlineStr"/>
-      <c r="L69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001055] Tussenbericht vragen Bruin en Verhoef over Steeds meer vervuilde woningen in Rotterdam: &amp;#39;Mensen zijn bang erop afgerekend te worden&amp;#39;</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/c8013401-a09a-4d02-9c64-8c81c76bed10?documentId=07d1f586-7af1-40de-a734-5f693a6ed5c6</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001306] Beantwoording vragen Bruin en Verhoef over Steeds meer vervuilde woningen in Rotterdam: &amp;#39;Mensen zijn bang erop afgerekend te worden</t>
+        </is>
+      </c>
+      <c r="M69" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/c17a4cfe-76d8-4fbe-bff1-da17d551b4cd?documentId=116f5064-6129-4f4d-ab9e-075188732e62</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O69" s="2" t="inlineStr"/>
+      <c r="P69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -3901,11 +4381,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/01ddceb8-7b27-4c0c-8306-a225ba5b1317?documentId=f2e494f1-54a6-4d20-affb-27a897ff8880</t>
         </is>
       </c>
-      <c r="J70" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J70" s="2" t="inlineStr"/>
       <c r="K70" s="2" t="inlineStr"/>
-      <c r="L70" s="2" t="inlineStr"/>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000925] Beantwoording vragen de Haan over Nieuw icoon van Rotterdam</t>
+        </is>
+      </c>
+      <c r="M70" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/5a5759ea-a2fa-4337-a9ba-bf984049dc16?documentId=8262cc1b-0f5b-4548-ab9b-20ce3b3b2cca</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O70" s="2" t="inlineStr"/>
+      <c r="P70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -3953,11 +4445,31 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/cfcc0026-7fc2-417e-ad7b-a842cb0b6cdb?documentId=0c6fca7c-d0a3-467e-8c9b-efe867cae975</t>
         </is>
       </c>
-      <c r="J71" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K71" s="2" t="inlineStr"/>
-      <c r="L71" s="2" t="inlineStr"/>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>[25bb009674] Tussenbericht vragen Abrahamse over dreigende stroomuitval</t>
+        </is>
+      </c>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/9104e786-3f10-4290-9748-30c2da35415c?documentId=3aac4dab-eb4e-4250-a626-fc52254fe557</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001128] Beantwoording vragen Abrahamse over Dreigende stroomuitval</t>
+        </is>
+      </c>
+      <c r="M71" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/c0eb8214-b0c8-45b1-907f-d04e5d11ff03?documentId=84c2cca5-3b39-4bb0-8766-c92bf7de2a97</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O71" s="2" t="inlineStr"/>
+      <c r="P71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4005,11 +4517,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/2ea444ab-fec3-4d0b-a935-8157c0fb2f8c?documentId=ea25d1ac-6119-4d6a-88c6-a86594c27539</t>
         </is>
       </c>
-      <c r="J72" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J72" s="2" t="inlineStr"/>
       <c r="K72" s="2" t="inlineStr"/>
-      <c r="L72" s="2" t="inlineStr"/>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000743] Beantwoording vragen Vicario en Nunnely over Krachtige meisjes verdienen eerlijke kansen</t>
+        </is>
+      </c>
+      <c r="M72" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/5bca2bee-a095-4aa1-ad3f-a26aad9614f3?documentId=46a5c202-0a6c-490a-9598-08be14c6b959</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O72" s="2" t="inlineStr"/>
+      <c r="P72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4057,11 +4581,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/cca7f5ea-1c05-444f-82da-0a75923f53c1?documentId=3e9df6c4-292c-4391-a0f7-7824680dea3c</t>
         </is>
       </c>
-      <c r="J73" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J73" s="2" t="inlineStr"/>
       <c r="K73" s="2" t="inlineStr"/>
-      <c r="L73" s="2" t="inlineStr"/>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000475] Beantwoording vragen Morko&amp;#231; en Kockelkoren over Je kan het dak op (met een zonnepaneel)!</t>
+        </is>
+      </c>
+      <c r="M73" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/3987cef2-46e8-4687-8eed-d2a1be87237d?documentId=cf8bce91-e0eb-47a6-893e-055d64898c19</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O73" s="2" t="inlineStr"/>
+      <c r="P73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4109,11 +4645,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/c75f6216-1fc8-40e0-8dc2-756d3c8e8416?documentId=ce6a8b6d-2b5e-4b19-84b2-351e0088f447</t>
         </is>
       </c>
-      <c r="J74" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J74" s="2" t="inlineStr"/>
       <c r="K74" s="2" t="inlineStr"/>
-      <c r="L74" s="2" t="inlineStr"/>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000426] Beantwoording vragen Morkoc en Van der Velden over Spoed: Woef Woef Blaf Blaf, Red Hondenspeeltuin Bello</t>
+        </is>
+      </c>
+      <c r="M74" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/1ded1401-b3a3-4c93-8fbf-fdbb99be23b3?documentId=89ba8ebe-f3ae-4b89-99f4-348bc774767b</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O74" s="2" t="inlineStr"/>
+      <c r="P74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4161,11 +4709,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/6e29c291-5bd1-474b-bec0-608f83ef63ab?documentId=d1462eae-01a4-4cad-aa6f-33e3d941eea2</t>
         </is>
       </c>
-      <c r="J75" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J75" s="2" t="inlineStr"/>
       <c r="K75" s="2" t="inlineStr"/>
-      <c r="L75" s="2" t="inlineStr"/>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000297] Beantwoording vragen Roskam over Kwaliteitsniveau van huwelijksvoltrekkingen door “Babs voor &amp;#233;&amp;#233;n dag”</t>
+        </is>
+      </c>
+      <c r="M75" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/f4b5f52c-e6b3-456d-b2e1-f25976f5a97c?documentId=b00ee828-279f-479d-bb94-43d1cdb6ff13</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O75" s="2" t="inlineStr"/>
+      <c r="P75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4209,11 +4769,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/99550f64-f76c-4abe-9f4e-46f0d4ab8786?documentId=b9cd48cb-4179-4f9a-8fd1-edcc4f6039f5</t>
         </is>
       </c>
-      <c r="J76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000360] Tussenbericht vragen Aafjes - Van Aalst over maagdenvliesoperaties in Rotterdam</t>
+        </is>
+      </c>
+      <c r="K76" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/aa115a7c-f289-4506-b95e-0721c721ed07?documentId=d919695d-776d-4c30-ad57-f97587a94893</t>
+        </is>
+      </c>
       <c r="L76" s="2" t="inlineStr"/>
+      <c r="M76" s="2" t="inlineStr"/>
+      <c r="N76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" s="2" t="inlineStr"/>
+      <c r="P76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4257,11 +4829,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/31bcd874-ad1f-4465-9e6c-c233720a0e36?documentId=9becf741-b617-435d-a750-c2d6f59a7c28</t>
         </is>
       </c>
-      <c r="J77" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J77" s="2" t="inlineStr"/>
       <c r="K77" s="2" t="inlineStr"/>
       <c r="L77" s="2" t="inlineStr"/>
+      <c r="M77" s="2" t="inlineStr"/>
+      <c r="N77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O77" s="2" t="inlineStr"/>
+      <c r="P77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4305,11 +4881,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/6be2ef77-5aef-40b8-bbbb-4c6d7c5add79?documentId=a0f78653-7431-4a96-9fa9-5f21905c3d56</t>
         </is>
       </c>
-      <c r="J78" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>[25bb009538] Tussenbericht vragen Akhatab en Dahoe over Toegankelijke openbare toiletten voor rolstoelgebruikers in Rotterdam</t>
+        </is>
+      </c>
+      <c r="K78" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/9e5335a1-a449-4b29-8b87-85803e3b2d30?documentId=0a71f9fb-a717-45fb-b56e-8d5a6e30c568</t>
+        </is>
+      </c>
       <c r="L78" s="2" t="inlineStr"/>
+      <c r="M78" s="2" t="inlineStr"/>
+      <c r="N78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O78" s="2" t="inlineStr"/>
+      <c r="P78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -4353,11 +4941,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/0e5b0eb6-be79-4b97-929f-9c334877bdae?documentId=1838908a-9c99-4976-ac90-dbb89236f684</t>
         </is>
       </c>
-      <c r="J79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001408] Tussenbericht vragen Van der Velden over Zorgonthouding bij huisdieren door financi&amp;#235;le problemen en inzet dierenpolitie</t>
+        </is>
+      </c>
+      <c r="K79" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/b92f9df9-b20c-42c3-8129-380379c9e972?documentId=e7e0d5d4-c87f-4749-b963-0ecec57a16e7</t>
+        </is>
+      </c>
       <c r="L79" s="2" t="inlineStr"/>
+      <c r="M79" s="2" t="inlineStr"/>
+      <c r="N79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O79" s="2" t="inlineStr"/>
+      <c r="P79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -4405,11 +5005,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/34906ee9-c03a-499b-9dbe-8c1c813eb71e?documentId=6d6ee18b-78f9-4664-9864-09288e44d8af</t>
         </is>
       </c>
-      <c r="J80" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J80" s="2" t="inlineStr"/>
       <c r="K80" s="2" t="inlineStr"/>
-      <c r="L80" s="2" t="inlineStr"/>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000900] Beantwoording vragen Aafjes - van Aalst over Agressie tegen zorgpersoneel</t>
+        </is>
+      </c>
+      <c r="M80" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/d64a04c8-5dda-4097-a08d-00620fca494a?documentId=11516ba6-c37c-4303-8363-fb57f8ff258c</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O80" s="2" t="inlineStr"/>
+      <c r="P80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -4457,11 +5069,31 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/6920a27c-58c1-4307-bca0-96307d3e0530?documentId=4fcba6fa-045e-4597-a0a8-80fa25dbe6f6</t>
         </is>
       </c>
-      <c r="J81" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K81" s="2" t="inlineStr"/>
-      <c r="L81" s="2" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000072] Tussenbericht vragen Nunnely over (Gratis) leermiddelen voor mbo-studenten</t>
+        </is>
+      </c>
+      <c r="K81" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/cd8dadee-6ddd-4f85-8a1e-19aab691f833?documentId=43f2a162-47ea-478a-aaca-6a313a0d3d89</t>
+        </is>
+      </c>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001108] Beantwoording vragen Nunnely over (Gratis) leermiddelen voor mbo-studenten</t>
+        </is>
+      </c>
+      <c r="M81" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/651d814f-4e69-4cac-b708-5d1d1768e354?documentId=45a6818a-36bb-4dc0-8641-fc5299ccf0e4</t>
+        </is>
+      </c>
+      <c r="N81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O81" s="2" t="inlineStr"/>
+      <c r="P81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -4505,11 +5137,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/8cc4bd8c-f203-41e6-92a6-15c98454050c?documentId=7d33ab8b-2b0f-460a-86f1-639934a60c83</t>
         </is>
       </c>
-      <c r="J82" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J82" s="2" t="inlineStr"/>
       <c r="K82" s="2" t="inlineStr"/>
       <c r="L82" s="2" t="inlineStr"/>
+      <c r="M82" s="2" t="inlineStr"/>
+      <c r="N82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O82" s="2" t="inlineStr"/>
+      <c r="P82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -4553,11 +5189,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/493d1cdc-ed38-4546-bc67-109c294f2c95?documentId=1ae00564-2ab8-4eb0-ada3-dcbfa87764d3</t>
         </is>
       </c>
-      <c r="J83" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J83" s="2" t="inlineStr"/>
       <c r="K83" s="2" t="inlineStr"/>
       <c r="L83" s="2" t="inlineStr"/>
+      <c r="M83" s="2" t="inlineStr"/>
+      <c r="N83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O83" s="2" t="inlineStr"/>
+      <c r="P83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -4605,11 +5245,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/b0ad8655-c71b-4e1a-9856-3cae41c5a74b?documentId=a85381fa-0ae7-4d2d-bbf4-569b87181858</t>
         </is>
       </c>
-      <c r="J84" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J84" s="2" t="inlineStr"/>
       <c r="K84" s="2" t="inlineStr"/>
-      <c r="L84" s="2" t="inlineStr"/>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000253] Beantwoording vragen Van Wifferen over de wind op het dak hebben</t>
+        </is>
+      </c>
+      <c r="M84" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/1074d268-25f3-4b91-b8ca-bfd17e6c2b5f?documentId=06a57916-85f6-4225-8366-eef25a312c6d</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O84" s="2" t="inlineStr"/>
+      <c r="P84" s="2" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -4653,11 +5305,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/5c26aa43-8027-4fbb-9f2b-25207bd2e62c?documentId=cd5ec550-51d3-483e-8cef-8b924c53eaba</t>
         </is>
       </c>
-      <c r="J85" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J85" s="2" t="inlineStr"/>
       <c r="K85" s="2" t="inlineStr"/>
       <c r="L85" s="2" t="inlineStr"/>
+      <c r="M85" s="2" t="inlineStr"/>
+      <c r="N85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O85" s="2" t="inlineStr"/>
+      <c r="P85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -4701,11 +5357,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/1fbfa86d-4ae9-4a92-8c26-242c6a3f4ba4?documentId=10df9e1d-c550-4381-8154-fac1a5ffc86e</t>
         </is>
       </c>
-      <c r="J86" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J86" s="2" t="inlineStr"/>
       <c r="K86" s="2" t="inlineStr"/>
       <c r="L86" s="2" t="inlineStr"/>
+      <c r="M86" s="2" t="inlineStr"/>
+      <c r="N86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O86" s="2" t="inlineStr"/>
+      <c r="P86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -4753,11 +5413,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/2671001d-10dd-4e5c-92b5-3f336bd8df88?documentId=9c12047e-de6f-44d6-b14e-1060b6e1e677</t>
         </is>
       </c>
-      <c r="J87" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J87" s="2" t="inlineStr"/>
       <c r="K87" s="2" t="inlineStr"/>
-      <c r="L87" s="2" t="inlineStr"/>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001056] Beantwoording vragen Kockelkoren en de Bruijn over Vraag door, wees dakloosheid voor</t>
+        </is>
+      </c>
+      <c r="M87" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/67c120e1-479f-4ac9-9b3c-cb2a73e1fb2c?documentId=691357fc-900e-4472-9f73-b188d052fbb4</t>
+        </is>
+      </c>
+      <c r="N87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O87" s="2" t="inlineStr"/>
+      <c r="P87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -4805,11 +5477,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/f6340dc6-cfc7-4379-8f7e-8a92d1179432?documentId=e2d745f1-a59a-49b0-b2de-00df756b0da0</t>
         </is>
       </c>
-      <c r="J88" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J88" s="2" t="inlineStr"/>
       <c r="K88" s="2" t="inlineStr"/>
-      <c r="L88" s="2" t="inlineStr"/>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001391] Beantwoording vragen van Groningen over Fatbike-intimidatie in parken en bij sportclubs: welke maatregelen volgen</t>
+        </is>
+      </c>
+      <c r="M88" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/6482f5f6-f105-45b6-9df8-538c0b7e9834?documentId=5c0a2381-01b0-4269-90f4-1fc5fad9ce63</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O88" s="2" t="inlineStr"/>
+      <c r="P88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -4857,11 +5541,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/5f32798c-e445-4a45-aa59-881ef2a50861?documentId=8d10ac2e-4cbd-4e78-8da5-ff153be788d3</t>
         </is>
       </c>
-      <c r="J89" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J89" s="2" t="inlineStr"/>
       <c r="K89" s="2" t="inlineStr"/>
-      <c r="L89" s="2" t="inlineStr"/>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000696] Beantwoording vragen Balcha over aanbevelingen WODC - rapport &amp;#39;Werkverandering onder sekswerkers&amp;#39;</t>
+        </is>
+      </c>
+      <c r="M89" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/88f59dcb-8af3-459c-bc79-ebb13a3c6119?documentId=5da58895-2f8d-44c5-aa0a-eb3e6708182a</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O89" s="2" t="inlineStr"/>
+      <c r="P89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -4909,11 +5605,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/52ba1420-e399-4c51-a8f2-7d540f77b713?documentId=adb547d4-4fbf-4f63-a18d-32f11749aa52</t>
         </is>
       </c>
-      <c r="J90" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J90" s="2" t="inlineStr"/>
       <c r="K90" s="2" t="inlineStr"/>
-      <c r="L90" s="2" t="inlineStr"/>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000310] Beantwoording vragen Leewis over Geef ruimte aan sport in Rotterdam</t>
+        </is>
+      </c>
+      <c r="M90" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/59f1791f-6f42-4012-91e9-449a47394102?documentId=a2f626c1-9871-4b52-9381-9e23ea8e283c</t>
+        </is>
+      </c>
+      <c r="N90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O90" s="2" t="inlineStr"/>
+      <c r="P90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -4961,11 +5669,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/a6dbbd6e-d346-453a-be2c-9f88780218c7?documentId=732fea83-f6ad-40ae-8e0b-6fe5454a9e60</t>
         </is>
       </c>
-      <c r="J91" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J91" s="2" t="inlineStr"/>
       <c r="K91" s="2" t="inlineStr"/>
-      <c r="L91" s="2" t="inlineStr"/>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t>[25bb009238] beantwoording vragen van Dommelen over verdichting Sportdorp</t>
+        </is>
+      </c>
+      <c r="M91" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/b8c7c638-8b99-4a25-8f64-4e5948e874bf?documentId=bfe0519d-5506-4106-8511-e1f8dd887b18</t>
+        </is>
+      </c>
+      <c r="N91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O91" s="2" t="inlineStr"/>
+      <c r="P91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -5013,11 +5733,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/ed956046-459c-4ce8-b28f-03fdcb503ea2?documentId=9499586b-b15c-4940-9713-ad49494f39ef</t>
         </is>
       </c>
-      <c r="J92" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J92" s="2" t="inlineStr"/>
       <c r="K92" s="2" t="inlineStr"/>
-      <c r="L92" s="2" t="inlineStr"/>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>[26bb001234] Beantwoording vragen Koster en Van Aalst over Subsidieverlening Huizen van de Wijk</t>
+        </is>
+      </c>
+      <c r="M92" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/ab289465-3396-4f45-bdc3-da98ed7e816a?documentId=4fd406dd-e8ad-473a-ac05-a32e3b3af4f9</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O92" s="2" t="inlineStr"/>
+      <c r="P92" s="2" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -5061,11 +5793,15 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/f2eee099-7628-4b21-80ab-fc2892bd14eb?documentId=c53d20fa-d84f-4397-8bf3-2c6ff439b4c6</t>
         </is>
       </c>
-      <c r="J93" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J93" s="2" t="inlineStr"/>
       <c r="K93" s="2" t="inlineStr"/>
       <c r="L93" s="2" t="inlineStr"/>
+      <c r="M93" s="2" t="inlineStr"/>
+      <c r="N93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O93" s="2" t="inlineStr"/>
+      <c r="P93" s="2" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -5113,11 +5849,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/1c703c4b-7973-41d1-a006-c2bf8b794751?documentId=f7dc9980-25c5-4567-9901-4f924c41880a</t>
         </is>
       </c>
-      <c r="J94" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J94" s="2" t="inlineStr"/>
       <c r="K94" s="2" t="inlineStr"/>
-      <c r="L94" s="2" t="inlineStr"/>
+      <c r="L94" s="2" t="inlineStr">
+        <is>
+          <t>[25bb009465] Beantwoording vragen van Wifferen over Malafide verkopers thuisbatterijen</t>
+        </is>
+      </c>
+      <c r="M94" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/9f99648b-f296-4adf-b380-34555a5b92de?documentId=d1f8204c-e5ea-455c-9605-b6ec5a73304e</t>
+        </is>
+      </c>
+      <c r="N94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O94" s="2" t="inlineStr"/>
+      <c r="P94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -5165,11 +5913,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/b5b32a88-c797-4184-854a-72abaac1912f?documentId=6d925ba5-57f0-4ce1-a42a-b6f1530df79a</t>
         </is>
       </c>
-      <c r="J95" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J95" s="2" t="inlineStr"/>
       <c r="K95" s="2" t="inlineStr"/>
-      <c r="L95" s="2" t="inlineStr"/>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000831] Beantwoording vragen Bruin en Verhoef over Veiligheid balkons en galerijen bij Rotterdamse flats naar aanleiding van recente gebreken in Zeist</t>
+        </is>
+      </c>
+      <c r="M95" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/828e1655-3e8e-4e38-a7a7-ea0b63552fc1?documentId=577ecc3f-d654-46e9-a505-49931aba7122</t>
+        </is>
+      </c>
+      <c r="N95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O95" s="2" t="inlineStr"/>
+      <c r="P95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -5217,11 +5977,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/7589c571-7470-412e-8c31-aadd04263ecf?documentId=f2973963-d8cd-4db1-829f-a56c1d8a9219</t>
         </is>
       </c>
-      <c r="J96" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J96" s="2" t="inlineStr"/>
       <c r="K96" s="2" t="inlineStr"/>
-      <c r="L96" s="2" t="inlineStr"/>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000636] Beantwoording vragen Yildirim en Coskun over Het is tijd voor &amp;#233;chte duidelijkheid voor onze nutstuinders</t>
+        </is>
+      </c>
+      <c r="M96" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/8a731f04-9daa-4b04-a16d-744db51d4aa8?documentId=31d90ba4-c8c3-442e-aef9-1b9879c28dd0</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O96" s="2" t="inlineStr"/>
+      <c r="P96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -5265,11 +6037,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/e864923d-5b1b-46af-94da-11df2d66279b?documentId=de0dd704-4439-4a9b-9fff-95b39e39b8cb</t>
         </is>
       </c>
-      <c r="J97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K97" s="2" t="inlineStr"/>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>[25bb009267] Tussenbericht vragen Kind over Tijd voor echt openbaar toegankelijke toiletten</t>
+        </is>
+      </c>
+      <c r="K97" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/138d5f3d-3834-4c27-9765-c81fee237e45?documentId=18fd6e92-c1ff-429e-9dbb-63404d20d51d</t>
+        </is>
+      </c>
       <c r="L97" s="2" t="inlineStr"/>
+      <c r="M97" s="2" t="inlineStr"/>
+      <c r="N97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O97" s="2" t="inlineStr"/>
+      <c r="P97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -5313,11 +6097,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/eacda233-f444-49b1-befe-cd870bd4ad77?documentId=76ca2dab-966d-45de-a2c4-88ca23ffcd45</t>
         </is>
       </c>
-      <c r="J98" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K98" s="2" t="inlineStr"/>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>[25bb009018] Tussenbericht vragen van Campenhout over de uitbreiding en toepassing van de discriminerende Rotterdamwet</t>
+        </is>
+      </c>
+      <c r="K98" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/50f582a2-96ff-4aa5-8bd6-5873862b4d5a?documentId=18ad2053-63e0-4a02-a098-f1978ac07783</t>
+        </is>
+      </c>
       <c r="L98" s="2" t="inlineStr"/>
+      <c r="M98" s="2" t="inlineStr"/>
+      <c r="N98" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O98" s="2" t="inlineStr"/>
+      <c r="P98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -5365,11 +6161,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/13001bb7-76a0-4877-8992-afd721b58502?documentId=a6c350e9-abce-43a9-8ca7-2bf7b95b1cbe</t>
         </is>
       </c>
-      <c r="J99" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J99" s="2" t="inlineStr"/>
       <c r="K99" s="2" t="inlineStr"/>
-      <c r="L99" s="2" t="inlineStr"/>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>[25bb009458] Beantwoording vragen De Bruijn en Yildirim over Kansen voor statushouders in techniek en haven</t>
+        </is>
+      </c>
+      <c r="M99" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/bee49fb1-414a-4d8a-bc86-1b8055b95235?documentId=b23024c9-5b7d-41f0-8a6f-0ec96917fe45</t>
+        </is>
+      </c>
+      <c r="N99" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O99" s="2" t="inlineStr"/>
+      <c r="P99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -5417,11 +6225,23 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/b02cee96-4fb9-4713-88af-22baf097f9ec?documentId=5366c995-5735-4c4e-84d8-612b6d564413</t>
         </is>
       </c>
-      <c r="J100" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J100" s="2" t="inlineStr"/>
       <c r="K100" s="2" t="inlineStr"/>
-      <c r="L100" s="2" t="inlineStr"/>
+      <c r="L100" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000321] Beantwoording vragen Nunnely over De toekomst van onze Rotterdamse kunstacademie met aanvulling</t>
+        </is>
+      </c>
+      <c r="M100" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/4249f0fa-074d-4469-b1d6-aa8f94d7b31c?documentId=5b6aa7d3-da19-491b-8ed5-4e310861ce7a</t>
+        </is>
+      </c>
+      <c r="N100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O100" s="2" t="inlineStr"/>
+      <c r="P100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -5469,14 +6289,26 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/3949fc08-614a-410c-83f4-b588e45ce650?documentId=b0aa663f-64d6-44d3-8bb5-34e09dcb10d5</t>
         </is>
       </c>
-      <c r="J101" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J101" s="2" t="inlineStr"/>
       <c r="K101" s="2" t="inlineStr"/>
-      <c r="L101" s="2" t="inlineStr"/>
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>[26bb000244] Beantwoording vragen Vicario over van tevredenheid, naar resultaat</t>
+        </is>
+      </c>
+      <c r="M101" s="3" t="inlineStr">
+        <is>
+          <t>https://gemeenteraad.rotterdam.nl/Reports/Document/b7c77fd5-ba28-47cb-88fe-ef555d9f6aee?documentId=5caceb41-0677-4aca-b3f0-4dbafd1532dc</t>
+        </is>
+      </c>
+      <c r="N101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O101" s="2" t="inlineStr"/>
+      <c r="P101" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L101"/>
+  <autoFilter ref="A1:P101"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
@@ -5496,88 +6328,123 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I73" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I86" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I87" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I88" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I89" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I90" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I91" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I93" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I94" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I98" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I73" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I86" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I87" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I88" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I89" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M89" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I90" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M90" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I91" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I93" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I94" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M94" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M95" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M96" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I98" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M99" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M100" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I101" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M101" r:id="rId135"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Verwijder overbodige kolom 'Aantal bijlagen'
Bijlagen komen niet voor bij schriftelijke vragen; de kolom
was altijd 0. De kolom 'Bijlagen' (met namen) volstaat.

https://claude.ai/code/session_01Pt5DG8UgHAMFs55hwQTGmN
</commit_message>
<xml_diff>
--- a/schriftelijke_vragen.xlsx
+++ b/schriftelijke_vragen.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Schriftelijke vragen" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schriftelijke vragen'!$A$1:$P$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schriftelijke vragen'!$A$1:$O$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P101"/>
+  <dimension ref="A1:O101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -472,9 +472,8 @@
     <col width="50" customWidth="1" min="11" max="11"/>
     <col width="80" customWidth="1" min="12" max="12"/>
     <col width="50" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="100" customWidth="1" min="14" max="14"/>
     <col width="100" customWidth="1" min="15" max="15"/>
-    <col width="100" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -545,15 +544,10 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Aantal bijlagen</t>
+          <t>Bijlagen</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Bijlagen</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Bijlage URLs</t>
         </is>
@@ -605,11 +599,8 @@
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -657,11 +648,8 @@
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N3" s="2" t="inlineStr"/>
       <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -709,11 +697,8 @@
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N4" s="2" t="inlineStr"/>
       <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -761,11 +746,8 @@
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N5" s="2" t="inlineStr"/>
       <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -813,11 +795,8 @@
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N6" s="2" t="inlineStr"/>
       <c r="O6" s="2" t="inlineStr"/>
-      <c r="P6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -865,11 +844,8 @@
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N7" s="2" t="inlineStr"/>
       <c r="O7" s="2" t="inlineStr"/>
-      <c r="P7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -917,11 +893,8 @@
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N8" s="2" t="inlineStr"/>
       <c r="O8" s="2" t="inlineStr"/>
-      <c r="P8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -969,11 +942,8 @@
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
-      <c r="N9" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N9" s="2" t="inlineStr"/>
       <c r="O9" s="2" t="inlineStr"/>
-      <c r="P9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1021,11 +991,8 @@
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N10" s="2" t="inlineStr"/>
       <c r="O10" s="2" t="inlineStr"/>
-      <c r="P10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1073,11 +1040,8 @@
       <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
-      <c r="N11" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N11" s="2" t="inlineStr"/>
       <c r="O11" s="2" t="inlineStr"/>
-      <c r="P11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1125,11 +1089,8 @@
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N12" s="2" t="inlineStr"/>
       <c r="O12" s="2" t="inlineStr"/>
-      <c r="P12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1177,11 +1138,8 @@
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr"/>
-      <c r="N13" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N13" s="2" t="inlineStr"/>
       <c r="O13" s="2" t="inlineStr"/>
-      <c r="P13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1229,11 +1187,8 @@
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
-      <c r="N14" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="2" t="inlineStr"/>
-      <c r="P14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1281,11 +1236,8 @@
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr"/>
-      <c r="N15" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="2" t="inlineStr"/>
-      <c r="P15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1333,11 +1285,8 @@
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr"/>
-      <c r="P16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1385,11 +1334,8 @@
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
-      <c r="N17" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N17" s="2" t="inlineStr"/>
       <c r="O17" s="2" t="inlineStr"/>
-      <c r="P17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1437,11 +1383,8 @@
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
-      <c r="N18" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr"/>
-      <c r="P18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1501,11 +1444,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/c523cec4-6c8b-4433-8d67-51c5dd932fb0?documentId=42d17a26-9d7c-403b-bd5d-89a63aa6f585</t>
         </is>
       </c>
-      <c r="N19" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr"/>
-      <c r="P19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1553,11 +1493,8 @@
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
-      <c r="N20" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr"/>
-      <c r="P20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1605,11 +1542,8 @@
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr"/>
-      <c r="N21" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N21" s="2" t="inlineStr"/>
       <c r="O21" s="2" t="inlineStr"/>
-      <c r="P21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1657,11 +1591,8 @@
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N22" s="2" t="inlineStr"/>
       <c r="O22" s="2" t="inlineStr"/>
-      <c r="P22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1709,11 +1640,8 @@
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
-      <c r="N23" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N23" s="2" t="inlineStr"/>
       <c r="O23" s="2" t="inlineStr"/>
-      <c r="P23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1761,11 +1689,8 @@
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N24" s="2" t="inlineStr"/>
       <c r="O24" s="2" t="inlineStr"/>
-      <c r="P24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1813,11 +1738,8 @@
       <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr"/>
-      <c r="N25" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N25" s="2" t="inlineStr"/>
       <c r="O25" s="2" t="inlineStr"/>
-      <c r="P25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1865,11 +1787,8 @@
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N26" s="2" t="inlineStr"/>
       <c r="O26" s="2" t="inlineStr"/>
-      <c r="P26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1917,11 +1836,8 @@
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
-      <c r="N27" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N27" s="2" t="inlineStr"/>
       <c r="O27" s="2" t="inlineStr"/>
-      <c r="P27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1969,11 +1885,8 @@
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr"/>
-      <c r="P28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2021,11 +1934,8 @@
       <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
-      <c r="N29" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr"/>
-      <c r="P29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2073,11 +1983,8 @@
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
-      <c r="N30" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="2" t="inlineStr"/>
-      <c r="P30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2133,11 +2040,8 @@
       </c>
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
-      <c r="N31" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N31" s="2" t="inlineStr"/>
       <c r="O31" s="2" t="inlineStr"/>
-      <c r="P31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2185,11 +2089,8 @@
       <c r="K32" s="2" t="inlineStr"/>
       <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="2" t="inlineStr"/>
-      <c r="P32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2249,11 +2150,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/483fe85d-56c8-4ff0-a03e-e16eb94edd62?documentId=38d41caf-8e52-4c28-8f17-37ac4246c3b8</t>
         </is>
       </c>
-      <c r="N33" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N33" s="2" t="inlineStr"/>
       <c r="O33" s="2" t="inlineStr"/>
-      <c r="P33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2301,11 +2199,8 @@
       <c r="K34" s="2" t="inlineStr"/>
       <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N34" s="2" t="inlineStr"/>
       <c r="O34" s="2" t="inlineStr"/>
-      <c r="P34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2353,11 +2248,8 @@
       <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="2" t="inlineStr"/>
       <c r="M35" s="2" t="inlineStr"/>
-      <c r="N35" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N35" s="2" t="inlineStr"/>
       <c r="O35" s="2" t="inlineStr"/>
-      <c r="P35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2405,11 +2297,8 @@
       <c r="K36" s="2" t="inlineStr"/>
       <c r="L36" s="2" t="inlineStr"/>
       <c r="M36" s="2" t="inlineStr"/>
-      <c r="N36" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N36" s="2" t="inlineStr"/>
       <c r="O36" s="2" t="inlineStr"/>
-      <c r="P36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2457,11 +2346,8 @@
       <c r="K37" s="2" t="inlineStr"/>
       <c r="L37" s="2" t="inlineStr"/>
       <c r="M37" s="2" t="inlineStr"/>
-      <c r="N37" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N37" s="2" t="inlineStr"/>
       <c r="O37" s="2" t="inlineStr"/>
-      <c r="P37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2509,11 +2395,8 @@
       <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="2" t="inlineStr"/>
       <c r="M38" s="2" t="inlineStr"/>
-      <c r="N38" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N38" s="2" t="inlineStr"/>
       <c r="O38" s="2" t="inlineStr"/>
-      <c r="P38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2561,11 +2444,8 @@
       <c r="K39" s="2" t="inlineStr"/>
       <c r="L39" s="2" t="inlineStr"/>
       <c r="M39" s="2" t="inlineStr"/>
-      <c r="N39" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N39" s="2" t="inlineStr"/>
       <c r="O39" s="2" t="inlineStr"/>
-      <c r="P39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2621,11 +2501,8 @@
       </c>
       <c r="L40" s="2" t="inlineStr"/>
       <c r="M40" s="2" t="inlineStr"/>
-      <c r="N40" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N40" s="2" t="inlineStr"/>
       <c r="O40" s="2" t="inlineStr"/>
-      <c r="P40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2673,11 +2550,8 @@
       <c r="K41" s="2" t="inlineStr"/>
       <c r="L41" s="2" t="inlineStr"/>
       <c r="M41" s="2" t="inlineStr"/>
-      <c r="N41" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N41" s="2" t="inlineStr"/>
       <c r="O41" s="2" t="inlineStr"/>
-      <c r="P41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2737,11 +2611,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/f5471aff-ec53-4872-81e8-465dce85bcd1?documentId=ba36706a-6b27-4cf7-a010-965ea8499e00</t>
         </is>
       </c>
-      <c r="N42" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N42" s="2" t="inlineStr"/>
       <c r="O42" s="2" t="inlineStr"/>
-      <c r="P42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2801,11 +2672,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/06bf5008-a15d-4a89-9e8f-3a85e8fd2f8d?documentId=ad8fb670-d838-48e0-b2b6-a97124ca5c36</t>
         </is>
       </c>
-      <c r="N43" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N43" s="2" t="inlineStr"/>
       <c r="O43" s="2" t="inlineStr"/>
-      <c r="P43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2865,11 +2733,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/50844132-fce6-4823-b99d-563c6caff433?documentId=a18d25a1-61e4-4ce3-9642-74230d7a7a91</t>
         </is>
       </c>
-      <c r="N44" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N44" s="2" t="inlineStr"/>
       <c r="O44" s="2" t="inlineStr"/>
-      <c r="P44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2929,11 +2794,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/6b58d639-d3df-45f5-9b5b-1f7d737c2297?documentId=5b32e1f5-4056-484a-a989-a29296b91a17</t>
         </is>
       </c>
-      <c r="N45" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N45" s="2" t="inlineStr"/>
       <c r="O45" s="2" t="inlineStr"/>
-      <c r="P45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2989,11 +2851,8 @@
       </c>
       <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr"/>
-      <c r="N46" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N46" s="2" t="inlineStr"/>
       <c r="O46" s="2" t="inlineStr"/>
-      <c r="P46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3041,11 +2900,8 @@
       <c r="K47" s="2" t="inlineStr"/>
       <c r="L47" s="2" t="inlineStr"/>
       <c r="M47" s="2" t="inlineStr"/>
-      <c r="N47" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N47" s="2" t="inlineStr"/>
       <c r="O47" s="2" t="inlineStr"/>
-      <c r="P47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3093,11 +2949,8 @@
       <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr"/>
       <c r="M48" s="2" t="inlineStr"/>
-      <c r="N48" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N48" s="2" t="inlineStr"/>
       <c r="O48" s="2" t="inlineStr"/>
-      <c r="P48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3145,11 +2998,8 @@
       <c r="K49" s="2" t="inlineStr"/>
       <c r="L49" s="2" t="inlineStr"/>
       <c r="M49" s="2" t="inlineStr"/>
-      <c r="N49" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N49" s="2" t="inlineStr"/>
       <c r="O49" s="2" t="inlineStr"/>
-      <c r="P49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3205,11 +3055,8 @@
       </c>
       <c r="L50" s="2" t="inlineStr"/>
       <c r="M50" s="2" t="inlineStr"/>
-      <c r="N50" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N50" s="2" t="inlineStr"/>
       <c r="O50" s="2" t="inlineStr"/>
-      <c r="P50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3257,11 +3104,8 @@
       <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr"/>
       <c r="M51" s="2" t="inlineStr"/>
-      <c r="N51" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N51" s="2" t="inlineStr"/>
       <c r="O51" s="2" t="inlineStr"/>
-      <c r="P51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3309,11 +3153,8 @@
       <c r="K52" s="2" t="inlineStr"/>
       <c r="L52" s="2" t="inlineStr"/>
       <c r="M52" s="2" t="inlineStr"/>
-      <c r="N52" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N52" s="2" t="inlineStr"/>
       <c r="O52" s="2" t="inlineStr"/>
-      <c r="P52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3373,11 +3214,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/fd2e3566-e96d-4ed7-9bfd-18cec9127bfa?documentId=dfacf35d-15a4-4b14-bfaf-b5d1172c5b55</t>
         </is>
       </c>
-      <c r="N53" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N53" s="2" t="inlineStr"/>
       <c r="O53" s="2" t="inlineStr"/>
-      <c r="P53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3425,11 +3263,8 @@
       <c r="K54" s="2" t="inlineStr"/>
       <c r="L54" s="2" t="inlineStr"/>
       <c r="M54" s="2" t="inlineStr"/>
-      <c r="N54" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N54" s="2" t="inlineStr"/>
       <c r="O54" s="2" t="inlineStr"/>
-      <c r="P54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3489,11 +3324,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/27105e20-c966-486c-af9c-945f4daa4160?documentId=262b88a2-4655-4f80-ae2f-80a9a613f0f7</t>
         </is>
       </c>
-      <c r="N55" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N55" s="2" t="inlineStr"/>
       <c r="O55" s="2" t="inlineStr"/>
-      <c r="P55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3553,11 +3385,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/dfbad81c-7df9-4972-b3a3-341440b32a75?documentId=71e609c5-b3d2-4438-a6c3-1625ca87271c</t>
         </is>
       </c>
-      <c r="N56" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N56" s="2" t="inlineStr"/>
       <c r="O56" s="2" t="inlineStr"/>
-      <c r="P56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3613,11 +3442,8 @@
       </c>
       <c r="L57" s="2" t="inlineStr"/>
       <c r="M57" s="2" t="inlineStr"/>
-      <c r="N57" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N57" s="2" t="inlineStr"/>
       <c r="O57" s="2" t="inlineStr"/>
-      <c r="P57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3677,11 +3503,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/6f55d6a7-37cd-4a58-8b74-56fba1c4fa9f?documentId=5706c4e6-b86e-47cc-8f5e-5c95046cc443</t>
         </is>
       </c>
-      <c r="N58" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N58" s="2" t="inlineStr"/>
       <c r="O58" s="2" t="inlineStr"/>
-      <c r="P58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3729,11 +3552,8 @@
       <c r="K59" s="2" t="inlineStr"/>
       <c r="L59" s="2" t="inlineStr"/>
       <c r="M59" s="2" t="inlineStr"/>
-      <c r="N59" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N59" s="2" t="inlineStr"/>
       <c r="O59" s="2" t="inlineStr"/>
-      <c r="P59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3793,11 +3613,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/7f6770f4-cc2b-417e-b00b-08b8ad6aa267?documentId=fd6f9042-9612-43a0-a373-d3d1116d3a09</t>
         </is>
       </c>
-      <c r="N60" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N60" s="2" t="inlineStr"/>
       <c r="O60" s="2" t="inlineStr"/>
-      <c r="P60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3853,11 +3670,8 @@
       </c>
       <c r="L61" s="2" t="inlineStr"/>
       <c r="M61" s="2" t="inlineStr"/>
-      <c r="N61" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N61" s="2" t="inlineStr"/>
       <c r="O61" s="2" t="inlineStr"/>
-      <c r="P61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3905,11 +3719,8 @@
       <c r="K62" s="2" t="inlineStr"/>
       <c r="L62" s="2" t="inlineStr"/>
       <c r="M62" s="2" t="inlineStr"/>
-      <c r="N62" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N62" s="2" t="inlineStr"/>
       <c r="O62" s="2" t="inlineStr"/>
-      <c r="P62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3969,11 +3780,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/c8eb5f8f-8f03-4aa1-934d-9b047a90881e?documentId=eaf65cca-3e07-41c8-bf49-1d82be382c3d</t>
         </is>
       </c>
-      <c r="N63" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N63" s="2" t="inlineStr"/>
       <c r="O63" s="2" t="inlineStr"/>
-      <c r="P63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4029,11 +3837,8 @@
       </c>
       <c r="L64" s="2" t="inlineStr"/>
       <c r="M64" s="2" t="inlineStr"/>
-      <c r="N64" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N64" s="2" t="inlineStr"/>
       <c r="O64" s="2" t="inlineStr"/>
-      <c r="P64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4089,11 +3894,8 @@
       </c>
       <c r="L65" s="2" t="inlineStr"/>
       <c r="M65" s="2" t="inlineStr"/>
-      <c r="N65" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N65" s="2" t="inlineStr"/>
       <c r="O65" s="2" t="inlineStr"/>
-      <c r="P65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4141,11 +3943,8 @@
       <c r="K66" s="2" t="inlineStr"/>
       <c r="L66" s="2" t="inlineStr"/>
       <c r="M66" s="2" t="inlineStr"/>
-      <c r="N66" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N66" s="2" t="inlineStr"/>
       <c r="O66" s="2" t="inlineStr"/>
-      <c r="P66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4193,11 +3992,8 @@
       <c r="K67" s="2" t="inlineStr"/>
       <c r="L67" s="2" t="inlineStr"/>
       <c r="M67" s="2" t="inlineStr"/>
-      <c r="N67" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N67" s="2" t="inlineStr"/>
       <c r="O67" s="2" t="inlineStr"/>
-      <c r="P67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4257,11 +4053,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/ae4a7388-ce55-470b-88d5-6250ea72a4c9?documentId=13ac84aa-4119-4cc0-bf06-853fcb5108cd</t>
         </is>
       </c>
-      <c r="N68" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N68" s="2" t="inlineStr"/>
       <c r="O68" s="2" t="inlineStr"/>
-      <c r="P68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4329,11 +4122,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/c17a4cfe-76d8-4fbe-bff1-da17d551b4cd?documentId=116f5064-6129-4f4d-ab9e-075188732e62</t>
         </is>
       </c>
-      <c r="N69" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N69" s="2" t="inlineStr"/>
       <c r="O69" s="2" t="inlineStr"/>
-      <c r="P69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4393,11 +4183,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/5a5759ea-a2fa-4337-a9ba-bf984049dc16?documentId=8262cc1b-0f5b-4548-ab9b-20ce3b3b2cca</t>
         </is>
       </c>
-      <c r="N70" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N70" s="2" t="inlineStr"/>
       <c r="O70" s="2" t="inlineStr"/>
-      <c r="P70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4465,11 +4252,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/c0eb8214-b0c8-45b1-907f-d04e5d11ff03?documentId=84c2cca5-3b39-4bb0-8766-c92bf7de2a97</t>
         </is>
       </c>
-      <c r="N71" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N71" s="2" t="inlineStr"/>
       <c r="O71" s="2" t="inlineStr"/>
-      <c r="P71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4529,11 +4313,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/5bca2bee-a095-4aa1-ad3f-a26aad9614f3?documentId=46a5c202-0a6c-490a-9598-08be14c6b959</t>
         </is>
       </c>
-      <c r="N72" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N72" s="2" t="inlineStr"/>
       <c r="O72" s="2" t="inlineStr"/>
-      <c r="P72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4593,11 +4374,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/3987cef2-46e8-4687-8eed-d2a1be87237d?documentId=cf8bce91-e0eb-47a6-893e-055d64898c19</t>
         </is>
       </c>
-      <c r="N73" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N73" s="2" t="inlineStr"/>
       <c r="O73" s="2" t="inlineStr"/>
-      <c r="P73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4657,11 +4435,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/1ded1401-b3a3-4c93-8fbf-fdbb99be23b3?documentId=89ba8ebe-f3ae-4b89-99f4-348bc774767b</t>
         </is>
       </c>
-      <c r="N74" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N74" s="2" t="inlineStr"/>
       <c r="O74" s="2" t="inlineStr"/>
-      <c r="P74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4721,11 +4496,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/f4b5f52c-e6b3-456d-b2e1-f25976f5a97c?documentId=b00ee828-279f-479d-bb94-43d1cdb6ff13</t>
         </is>
       </c>
-      <c r="N75" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N75" s="2" t="inlineStr"/>
       <c r="O75" s="2" t="inlineStr"/>
-      <c r="P75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4781,11 +4553,8 @@
       </c>
       <c r="L76" s="2" t="inlineStr"/>
       <c r="M76" s="2" t="inlineStr"/>
-      <c r="N76" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N76" s="2" t="inlineStr"/>
       <c r="O76" s="2" t="inlineStr"/>
-      <c r="P76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4833,11 +4602,8 @@
       <c r="K77" s="2" t="inlineStr"/>
       <c r="L77" s="2" t="inlineStr"/>
       <c r="M77" s="2" t="inlineStr"/>
-      <c r="N77" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N77" s="2" t="inlineStr"/>
       <c r="O77" s="2" t="inlineStr"/>
-      <c r="P77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4893,11 +4659,8 @@
       </c>
       <c r="L78" s="2" t="inlineStr"/>
       <c r="M78" s="2" t="inlineStr"/>
-      <c r="N78" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N78" s="2" t="inlineStr"/>
       <c r="O78" s="2" t="inlineStr"/>
-      <c r="P78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -4953,11 +4716,8 @@
       </c>
       <c r="L79" s="2" t="inlineStr"/>
       <c r="M79" s="2" t="inlineStr"/>
-      <c r="N79" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N79" s="2" t="inlineStr"/>
       <c r="O79" s="2" t="inlineStr"/>
-      <c r="P79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -5017,11 +4777,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/d64a04c8-5dda-4097-a08d-00620fca494a?documentId=11516ba6-c37c-4303-8363-fb57f8ff258c</t>
         </is>
       </c>
-      <c r="N80" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N80" s="2" t="inlineStr"/>
       <c r="O80" s="2" t="inlineStr"/>
-      <c r="P80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5089,11 +4846,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/651d814f-4e69-4cac-b708-5d1d1768e354?documentId=45a6818a-36bb-4dc0-8641-fc5299ccf0e4</t>
         </is>
       </c>
-      <c r="N81" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N81" s="2" t="inlineStr"/>
       <c r="O81" s="2" t="inlineStr"/>
-      <c r="P81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5141,11 +4895,8 @@
       <c r="K82" s="2" t="inlineStr"/>
       <c r="L82" s="2" t="inlineStr"/>
       <c r="M82" s="2" t="inlineStr"/>
-      <c r="N82" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N82" s="2" t="inlineStr"/>
       <c r="O82" s="2" t="inlineStr"/>
-      <c r="P82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -5193,11 +4944,8 @@
       <c r="K83" s="2" t="inlineStr"/>
       <c r="L83" s="2" t="inlineStr"/>
       <c r="M83" s="2" t="inlineStr"/>
-      <c r="N83" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N83" s="2" t="inlineStr"/>
       <c r="O83" s="2" t="inlineStr"/>
-      <c r="P83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -5257,11 +5005,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/1074d268-25f3-4b91-b8ca-bfd17e6c2b5f?documentId=06a57916-85f6-4225-8366-eef25a312c6d</t>
         </is>
       </c>
-      <c r="N84" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N84" s="2" t="inlineStr"/>
       <c r="O84" s="2" t="inlineStr"/>
-      <c r="P84" s="2" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -5309,11 +5054,8 @@
       <c r="K85" s="2" t="inlineStr"/>
       <c r="L85" s="2" t="inlineStr"/>
       <c r="M85" s="2" t="inlineStr"/>
-      <c r="N85" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N85" s="2" t="inlineStr"/>
       <c r="O85" s="2" t="inlineStr"/>
-      <c r="P85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5361,11 +5103,8 @@
       <c r="K86" s="2" t="inlineStr"/>
       <c r="L86" s="2" t="inlineStr"/>
       <c r="M86" s="2" t="inlineStr"/>
-      <c r="N86" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N86" s="2" t="inlineStr"/>
       <c r="O86" s="2" t="inlineStr"/>
-      <c r="P86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -5425,11 +5164,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/67c120e1-479f-4ac9-9b3c-cb2a73e1fb2c?documentId=691357fc-900e-4472-9f73-b188d052fbb4</t>
         </is>
       </c>
-      <c r="N87" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N87" s="2" t="inlineStr"/>
       <c r="O87" s="2" t="inlineStr"/>
-      <c r="P87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5489,11 +5225,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/6482f5f6-f105-45b6-9df8-538c0b7e9834?documentId=5c0a2381-01b0-4269-90f4-1fc5fad9ce63</t>
         </is>
       </c>
-      <c r="N88" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N88" s="2" t="inlineStr"/>
       <c r="O88" s="2" t="inlineStr"/>
-      <c r="P88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -5553,11 +5286,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/88f59dcb-8af3-459c-bc79-ebb13a3c6119?documentId=5da58895-2f8d-44c5-aa0a-eb3e6708182a</t>
         </is>
       </c>
-      <c r="N89" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N89" s="2" t="inlineStr"/>
       <c r="O89" s="2" t="inlineStr"/>
-      <c r="P89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5617,11 +5347,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/59f1791f-6f42-4012-91e9-449a47394102?documentId=a2f626c1-9871-4b52-9381-9e23ea8e283c</t>
         </is>
       </c>
-      <c r="N90" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N90" s="2" t="inlineStr"/>
       <c r="O90" s="2" t="inlineStr"/>
-      <c r="P90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5681,11 +5408,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/b8c7c638-8b99-4a25-8f64-4e5948e874bf?documentId=bfe0519d-5506-4106-8511-e1f8dd887b18</t>
         </is>
       </c>
-      <c r="N91" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N91" s="2" t="inlineStr"/>
       <c r="O91" s="2" t="inlineStr"/>
-      <c r="P91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -5745,11 +5469,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/ab289465-3396-4f45-bdc3-da98ed7e816a?documentId=4fd406dd-e8ad-473a-ac05-a32e3b3af4f9</t>
         </is>
       </c>
-      <c r="N92" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N92" s="2" t="inlineStr"/>
       <c r="O92" s="2" t="inlineStr"/>
-      <c r="P92" s="2" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -5797,11 +5518,8 @@
       <c r="K93" s="2" t="inlineStr"/>
       <c r="L93" s="2" t="inlineStr"/>
       <c r="M93" s="2" t="inlineStr"/>
-      <c r="N93" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N93" s="2" t="inlineStr"/>
       <c r="O93" s="2" t="inlineStr"/>
-      <c r="P93" s="2" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -5861,11 +5579,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/9f99648b-f296-4adf-b380-34555a5b92de?documentId=d1f8204c-e5ea-455c-9605-b6ec5a73304e</t>
         </is>
       </c>
-      <c r="N94" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N94" s="2" t="inlineStr"/>
       <c r="O94" s="2" t="inlineStr"/>
-      <c r="P94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -5925,11 +5640,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/828e1655-3e8e-4e38-a7a7-ea0b63552fc1?documentId=577ecc3f-d654-46e9-a505-49931aba7122</t>
         </is>
       </c>
-      <c r="N95" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N95" s="2" t="inlineStr"/>
       <c r="O95" s="2" t="inlineStr"/>
-      <c r="P95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -5989,11 +5701,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/8a731f04-9daa-4b04-a16d-744db51d4aa8?documentId=31d90ba4-c8c3-442e-aef9-1b9879c28dd0</t>
         </is>
       </c>
-      <c r="N96" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N96" s="2" t="inlineStr"/>
       <c r="O96" s="2" t="inlineStr"/>
-      <c r="P96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -6049,11 +5758,8 @@
       </c>
       <c r="L97" s="2" t="inlineStr"/>
       <c r="M97" s="2" t="inlineStr"/>
-      <c r="N97" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N97" s="2" t="inlineStr"/>
       <c r="O97" s="2" t="inlineStr"/>
-      <c r="P97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -6109,11 +5815,8 @@
       </c>
       <c r="L98" s="2" t="inlineStr"/>
       <c r="M98" s="2" t="inlineStr"/>
-      <c r="N98" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N98" s="2" t="inlineStr"/>
       <c r="O98" s="2" t="inlineStr"/>
-      <c r="P98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -6173,11 +5876,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/bee49fb1-414a-4d8a-bc86-1b8055b95235?documentId=b23024c9-5b7d-41f0-8a6f-0ec96917fe45</t>
         </is>
       </c>
-      <c r="N99" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N99" s="2" t="inlineStr"/>
       <c r="O99" s="2" t="inlineStr"/>
-      <c r="P99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -6237,11 +5937,8 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/4249f0fa-074d-4469-b1d6-aa8f94d7b31c?documentId=5b6aa7d3-da19-491b-8ed5-4e310861ce7a</t>
         </is>
       </c>
-      <c r="N100" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N100" s="2" t="inlineStr"/>
       <c r="O100" s="2" t="inlineStr"/>
-      <c r="P100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -6301,14 +5998,11 @@
           <t>https://gemeenteraad.rotterdam.nl/Reports/Document/b7c77fd5-ba28-47cb-88fe-ef555d9f6aee?documentId=5caceb41-0677-4aca-b3f0-4dbafd1532dc</t>
         </is>
       </c>
-      <c r="N101" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="N101" s="2" t="inlineStr"/>
       <c r="O101" s="2" t="inlineStr"/>
-      <c r="P101" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P101"/>
+  <autoFilter ref="A1:O101"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>

</xml_diff>